<commit_message>
Per-package cost with materials, labor, fuel and ads per wash
Claude-Session: https://claude.ai/code/session_013XYEeoGyPbCxnWrxN9YYVu
</commit_message>
<xml_diff>
--- a/car-wash/finance/cost-per-wash-table.xlsx
+++ b/car-wash/finance/cost-per-wash-table.xlsx
@@ -107,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -130,6 +130,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -141,7 +155,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -216,6 +230,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,348 +490,291 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" style="9" min="1" max="1"/>
-    <col width="15" customWidth="1" style="9" min="2" max="9"/>
+    <col width="18" customWidth="1" style="10" min="1" max="1"/>
+    <col width="13" customWidth="1" style="10" min="2" max="2"/>
+    <col width="13" customWidth="1" style="10" min="3" max="3"/>
+    <col width="13" customWidth="1" style="10" min="4" max="4"/>
+    <col width="13" customWidth="1" style="10" min="5" max="5"/>
+    <col width="13" customWidth="1" style="10" min="6" max="6"/>
+    <col width="13" customWidth="1" style="10" min="7" max="7"/>
+    <col width="13" customWidth="1" style="10" min="8" max="8"/>
+    <col width="13" customWidth="1" style="10" min="9" max="9"/>
+    <col width="13" customWidth="1" style="10" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="23.85" customHeight="1" s="10">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>الباقة</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>المواد للغسلة</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>العمال للغسلة</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>بنزين وكهرباء للغسلة</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>المواد</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>العامل</t>
+        </is>
+      </c>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>البنزين والكهرباء</t>
+        </is>
+      </c>
+      <c r="E1" s="26" t="inlineStr">
+        <is>
+          <t>الإعلانات</t>
+        </is>
+      </c>
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>التكلفة الكاملة</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>سعر صالون</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>ربح صالون</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>سعر جيب</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>ربح جيب</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="10">
-      <c r="A2" s="12" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>ببلز</t>
         </is>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="28">
         <f>'مواد الغسلة'!B11</f>
         <v/>
       </c>
-      <c r="C2" s="13">
-        <f>المدخلات!B2*المدخلات!B3/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="D2" s="13">
-        <f>المدخلات!B4*المدخلات!B5*52/12/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="E2" s="13">
-        <f>B2+C2+D2</f>
-        <v/>
-      </c>
-      <c r="F2" s="12" t="n">
+      <c r="C2" s="28">
+        <f>'المدخلات'!B2*'المدخلات'!B3/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="D2" s="28">
+        <f>'المدخلات'!B4*'المدخلات'!B5*52/12/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="E2" s="28">
+        <f>'المدخلات'!B18/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="F2" s="28">
+        <f>B2+C2+D2+E2</f>
+        <v/>
+      </c>
+      <c r="G2" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="G2" s="13">
-        <f>F2-E2</f>
-        <v/>
-      </c>
-      <c r="H2" s="12" t="n">
+      <c r="H2" s="28">
+        <f>G2-F2</f>
+        <v/>
+      </c>
+      <c r="I2" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="I2" s="13">
-        <f>H2-E2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="10">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="J2" s="28">
+        <f>I2-F2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>دبل ببلز</t>
         </is>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="28">
         <f>'مواد الغسلة'!C11</f>
         <v/>
       </c>
-      <c r="C3" s="13">
-        <f>المدخلات!B2*المدخلات!B3/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="D3" s="13">
-        <f>المدخلات!B4*المدخلات!B5*52/12/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="E3" s="13">
-        <f>B3+C3+D3</f>
-        <v/>
-      </c>
-      <c r="F3" s="12" t="n">
+      <c r="C3" s="28">
+        <f>'المدخلات'!B2*'المدخلات'!B3/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="D3" s="28">
+        <f>'المدخلات'!B4*'المدخلات'!B5*52/12/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="E3" s="28">
+        <f>'المدخلات'!B18/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="F3" s="28">
+        <f>B3+C3+D3+E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="G3" s="13">
-        <f>F3-E3</f>
-        <v/>
-      </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="28">
+        <f>G3-F3</f>
+        <v/>
+      </c>
+      <c r="I3" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="I3" s="13">
-        <f>H3-E3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="10">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="J3" s="28">
+        <f>I3-F3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>سوبر ببلز</t>
         </is>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="28">
         <f>'مواد الغسلة'!D11</f>
         <v/>
       </c>
-      <c r="C4" s="13">
-        <f>المدخلات!B2*المدخلات!B3/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="D4" s="13">
-        <f>المدخلات!B4*المدخلات!B5*52/12/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="E4" s="13">
-        <f>B4+C4+D4</f>
-        <v/>
-      </c>
-      <c r="F4" s="12" t="n">
+      <c r="C4" s="28">
+        <f>'المدخلات'!B2*'المدخلات'!B3/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="D4" s="28">
+        <f>'المدخلات'!B4*'المدخلات'!B5*52/12/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="E4" s="28">
+        <f>'المدخلات'!B18/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="F4" s="28">
+        <f>B4+C4+D4+E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="28" t="n">
         <v>15</v>
       </c>
-      <c r="G4" s="13">
-        <f>F4-E4</f>
-        <v/>
-      </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="28">
+        <f>G4-F4</f>
+        <v/>
+      </c>
+      <c r="I4" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="I4" s="13">
-        <f>H4-E4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="10">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="J4" s="28">
+        <f>I4-F4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>سوبر توب ببلز</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="28">
         <f>'مواد الغسلة'!E11</f>
         <v/>
       </c>
-      <c r="C5" s="13">
-        <f>المدخلات!B2*المدخلات!B3/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="D5" s="13">
-        <f>المدخلات!B4*المدخلات!B5*52/12/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="E5" s="13">
-        <f>B5+C5+D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="12" t="n">
+      <c r="C5" s="28">
+        <f>'المدخلات'!B2*'المدخلات'!B3/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="D5" s="28">
+        <f>'المدخلات'!B4*'المدخلات'!B5*52/12/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="E5" s="28">
+        <f>'المدخلات'!B18/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="F5" s="28">
+        <f>B5+C5+D5+E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="G5" s="13">
-        <f>F5-E5</f>
-        <v/>
-      </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="28">
+        <f>G5-F5</f>
+        <v/>
+      </c>
+      <c r="I5" s="28" t="n">
         <v>25</v>
       </c>
-      <c r="I5" s="13">
-        <f>H5-E5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="10">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="J5" s="28">
+        <f>I5-F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>سبشل ببلز</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="28">
         <f>'مواد الغسلة'!F11</f>
         <v/>
       </c>
-      <c r="C6" s="13">
-        <f>المدخلات!B2*المدخلات!B3/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="D6" s="13">
-        <f>المدخلات!B4*المدخلات!B5*52/12/(المدخلات!B5*المدخلات!B6*المدخلات!B7)</f>
-        <v/>
-      </c>
-      <c r="E6" s="13">
-        <f>B6+C6+D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="12" t="n">
+      <c r="C6" s="28">
+        <f>'المدخلات'!B2*'المدخلات'!B3/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="D6" s="28">
+        <f>'المدخلات'!B4*'المدخلات'!B5*52/12/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="E6" s="28">
+        <f>'المدخلات'!B18/('المدخلات'!B5*'المدخلات'!B6*'المدخلات'!B7)</f>
+        <v/>
+      </c>
+      <c r="F6" s="28">
+        <f>B6+C6+D6+E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="28" t="n">
         <v>35</v>
       </c>
-      <c r="G6" s="13">
-        <f>F6-E6</f>
-        <v/>
-      </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="28">
+        <f>G6-F6</f>
+        <v/>
+      </c>
+      <c r="I6" s="28" t="n">
         <v>40</v>
       </c>
-      <c r="I6" s="13">
-        <f>H6-E6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="10">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>الشهر (312 غسلة، توزيع 50/30/15/5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="10">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>الإيراد الشهري</t>
-        </is>
-      </c>
-      <c r="B9" s="15">
-        <f>312*(0.5*AVERAGE(F2,H2)+0.3*AVERAGE(F3,H3)+0.15*AVERAGE(F4,H4,F5,H5)+0.05*AVERAGE(F6,H6))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>المواد الشهرية</t>
-        </is>
-      </c>
-      <c r="B10" s="15">
-        <f>312*(0.5*B2+0.3*B3+0.15*AVERAGE(B4,B5)+0.05*B6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="10">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>العمال الشهرية</t>
-        </is>
-      </c>
-      <c r="B11" s="15">
-        <f>المدخلات!B2*المدخلات!B3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="10">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>البنزين والكهرباء الشهرية</t>
-        </is>
-      </c>
-      <c r="B12" s="15">
-        <f>المدخلات!B4*المدخلات!B5*52/12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="10">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>الإعلانات</t>
-        </is>
-      </c>
-      <c r="B13" s="15">
-        <f>المدخلات!B18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="10">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>إجمالي التكلفة الشهرية</t>
-        </is>
-      </c>
-      <c r="B14" s="15">
-        <f>B10+B11+B12+B13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="10">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>الربح الشهري</t>
-        </is>
-      </c>
-      <c r="B15" s="16">
-        <f>B9-B14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="10">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>نقطة التعادل (غسلات بالشهر)</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>ROUNDUP((B11+B12+B13)/((B9-B10)/312),0)</f>
-        <v/>
+      <c r="J6" s="28">
+        <f>I6-F6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>الملاحظة: كل قيمة هي تكلفة الغسلة الواحدة بالدينار. العامل والبنزين والإعلانات موزعة على الغسلات (312 بالشهر).</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>